<commit_message>
Playoffs final (Skybrook): Ethan High wins the 2026 championship
- Semifinal 1 (Front 9): Curtis Lynn def. Preston Stoner 4.5-3.5 (NET 35 vs 38)
- Semifinal 2: Ethan High advances - Charlotte Hayes forfeit
- Championship (Back 9): Ethan High def. Curtis Lynn 5-3 (NET 37 vs 39)
- 3rd Place: Preston Stoner - Charlotte Hayes forfeit

Final order: Ethan High, Curtis Lynn, Preston Stoner, Charlotte Hayes.
Dashboard Playoffs tab gets a champion banner, a forfeit note and a Final subtitle.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Score Calculator.xlsx
+++ b/Score Calculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imicompanies-my.sharepoint.com/personal/ehigh_iengtobuild_com/Documents/Documents/Golf League/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="11_F79F0194A688F399554C0C2CC307F263D8A13CD6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94C9C597-CF82-4441-B087-34D15CBB94D3}"/>
+  <xr:revisionPtr revIDLastSave="85" documentId="11_F79F0194A688F399554C0C2CC307F263D8A13CD6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B89AA4B-082D-4ADB-983C-16F6C04D1DAF}"/>
   <bookViews>
-    <workbookView xWindow="38295" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculator" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,6 @@
     <definedName name="Warrior_Golf_Club">Helper!$E$3:$E$5</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -478,7 +477,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -596,85 +595,76 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1176,16 +1166,16 @@
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J1" s="49" t="s">
-        <v>1</v>
-      </c>
-      <c r="K1" s="50"/>
-      <c r="L1" s="50"/>
-      <c r="M1" s="50"/>
+      <c r="J1" s="52" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="53"/>
+      <c r="L1" s="53"/>
+      <c r="M1" s="53"/>
     </row>
     <row r="2" spans="2:99" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>3</v>
@@ -1203,16 +1193,16 @@
         <v>7</v>
       </c>
       <c r="I2" s="5"/>
-      <c r="J2" s="47" t="str">
+      <c r="J2" s="66" t="str">
         <f>B8</f>
         <v>Curtis Lynn</v>
       </c>
-      <c r="K2" s="40"/>
-      <c r="L2" s="39" t="str">
+      <c r="K2" s="61"/>
+      <c r="L2" s="60" t="str">
         <f>B17</f>
-        <v>Alex Palmer</v>
-      </c>
-      <c r="M2" s="40"/>
+        <v>Ethan High</v>
+      </c>
+      <c r="M2" s="61"/>
     </row>
     <row r="3" spans="2:99" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B3" s="48" t="str">
@@ -1228,33 +1218,33 @@
       </c>
       <c r="E3" s="7">
         <f>SUM(F15:H15)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3" s="7">
         <f>SUM(I15:K15)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G3" s="7">
         <f>SUM(C15:K15)</f>
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H3" s="7">
         <f>SUM(C14:K14)</f>
-        <v>33</v>
-      </c>
-      <c r="J3" s="41">
+        <v>39</v>
+      </c>
+      <c r="J3" s="64">
         <f>SUM(D4:H4)</f>
-        <v>7</v>
-      </c>
-      <c r="K3" s="42"/>
-      <c r="L3" s="51">
+        <v>3</v>
+      </c>
+      <c r="K3" s="57"/>
+      <c r="L3" s="56">
         <f>SUM(D6:H6)</f>
-        <v>1</v>
-      </c>
-      <c r="M3" s="42"/>
+        <v>5</v>
+      </c>
+      <c r="M3" s="57"/>
     </row>
     <row r="4" spans="2:99" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="45"/>
+      <c r="B4" s="49"/>
       <c r="C4" s="8" t="s">
         <v>9</v>
       </c>
@@ -1268,25 +1258,25 @@
       </c>
       <c r="F4" s="9">
         <f>IF(F3&gt;F5,2,IF(F3=F5,1,0))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G4" s="9">
         <f>IF(G3&gt;G5,1,IF(G3=G5,0.5,0))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" s="9">
         <f>IF(H3&lt;H5,1,IF(H3=H5,0.5,0))</f>
-        <v>1</v>
-      </c>
-      <c r="J4" s="43"/>
-      <c r="K4" s="44"/>
-      <c r="L4" s="38"/>
-      <c r="M4" s="44"/>
+        <v>0</v>
+      </c>
+      <c r="J4" s="65"/>
+      <c r="K4" s="58"/>
+      <c r="L4" s="54"/>
+      <c r="M4" s="58"/>
     </row>
     <row r="5" spans="2:99" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B5" s="48" t="str">
         <f>L2</f>
-        <v>Alex Palmer</v>
+        <v>Ethan High</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>8</v>
@@ -1297,27 +1287,27 @@
       </c>
       <c r="E5" s="11">
         <f>SUM(F24:H24)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="11">
         <f>SUM(I24:K24)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G5" s="11">
         <f>SUM(C24:K24)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H5" s="11">
         <f>SUM(C23:K23)</f>
-        <v>48</v>
-      </c>
-      <c r="J5" s="45"/>
-      <c r="K5" s="46"/>
-      <c r="L5" s="50"/>
-      <c r="M5" s="46"/>
+        <v>37</v>
+      </c>
+      <c r="J5" s="49"/>
+      <c r="K5" s="59"/>
+      <c r="L5" s="53"/>
+      <c r="M5" s="59"/>
     </row>
     <row r="6" spans="2:99" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="45"/>
+      <c r="B6" s="49"/>
       <c r="C6" s="8" t="s">
         <v>9</v>
       </c>
@@ -1331,15 +1321,15 @@
       </c>
       <c r="F6" s="9">
         <f>IF(F5&gt;F3,2,IF(F5=F3,1,0))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G6" s="9">
         <f>IF(G5&gt;G3,1,IF(G5=G3,0.5,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6" s="9">
         <f>IF(H5&lt;H3,1,IF(H5=H3,0.5,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" s="12"/>
       <c r="K6" s="12"/>
@@ -1357,94 +1347,94 @@
       <c r="J7" s="12"/>
       <c r="K7" s="12"/>
       <c r="L7" s="12"/>
-      <c r="T7" s="64" t="s">
+      <c r="T7" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="U7" s="65"/>
-      <c r="V7" s="65"/>
-      <c r="W7" s="65"/>
-      <c r="X7" s="65"/>
-      <c r="Y7" s="65"/>
-      <c r="Z7" s="65"/>
-      <c r="AA7" s="65"/>
-      <c r="AB7" s="65"/>
-      <c r="AC7" s="65"/>
-      <c r="AD7" s="65"/>
-      <c r="AE7" s="65"/>
-      <c r="AF7" s="65"/>
-      <c r="AG7" s="65"/>
-      <c r="AH7" s="65"/>
-      <c r="AI7" s="65"/>
-      <c r="AJ7" s="65"/>
-      <c r="AK7" s="65"/>
-      <c r="AL7" s="65"/>
-      <c r="AM7" s="66"/>
-      <c r="AN7" s="64" t="s">
+      <c r="U7" s="50"/>
+      <c r="V7" s="50"/>
+      <c r="W7" s="50"/>
+      <c r="X7" s="50"/>
+      <c r="Y7" s="50"/>
+      <c r="Z7" s="50"/>
+      <c r="AA7" s="50"/>
+      <c r="AB7" s="50"/>
+      <c r="AC7" s="50"/>
+      <c r="AD7" s="50"/>
+      <c r="AE7" s="50"/>
+      <c r="AF7" s="50"/>
+      <c r="AG7" s="50"/>
+      <c r="AH7" s="50"/>
+      <c r="AI7" s="50"/>
+      <c r="AJ7" s="50"/>
+      <c r="AK7" s="50"/>
+      <c r="AL7" s="50"/>
+      <c r="AM7" s="51"/>
+      <c r="AN7" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="AO7" s="65"/>
-      <c r="AP7" s="65"/>
-      <c r="AQ7" s="65"/>
-      <c r="AR7" s="65"/>
-      <c r="AS7" s="65"/>
-      <c r="AT7" s="65"/>
-      <c r="AU7" s="65"/>
-      <c r="AV7" s="65"/>
-      <c r="AW7" s="65"/>
-      <c r="AX7" s="65"/>
-      <c r="AY7" s="65"/>
-      <c r="AZ7" s="65"/>
-      <c r="BA7" s="65"/>
-      <c r="BB7" s="65"/>
-      <c r="BC7" s="65"/>
-      <c r="BD7" s="65"/>
-      <c r="BE7" s="65"/>
-      <c r="BF7" s="65"/>
-      <c r="BG7" s="66"/>
-      <c r="BH7" s="64" t="s">
+      <c r="AO7" s="50"/>
+      <c r="AP7" s="50"/>
+      <c r="AQ7" s="50"/>
+      <c r="AR7" s="50"/>
+      <c r="AS7" s="50"/>
+      <c r="AT7" s="50"/>
+      <c r="AU7" s="50"/>
+      <c r="AV7" s="50"/>
+      <c r="AW7" s="50"/>
+      <c r="AX7" s="50"/>
+      <c r="AY7" s="50"/>
+      <c r="AZ7" s="50"/>
+      <c r="BA7" s="50"/>
+      <c r="BB7" s="50"/>
+      <c r="BC7" s="50"/>
+      <c r="BD7" s="50"/>
+      <c r="BE7" s="50"/>
+      <c r="BF7" s="50"/>
+      <c r="BG7" s="51"/>
+      <c r="BH7" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="BI7" s="65"/>
-      <c r="BJ7" s="67"/>
-      <c r="BK7" s="67"/>
-      <c r="BL7" s="67"/>
-      <c r="BM7" s="67"/>
-      <c r="BN7" s="67"/>
-      <c r="BO7" s="67"/>
-      <c r="BP7" s="67"/>
-      <c r="BQ7" s="67"/>
-      <c r="BR7" s="65"/>
-      <c r="BS7" s="65"/>
-      <c r="BT7" s="67"/>
-      <c r="BU7" s="67"/>
-      <c r="BV7" s="67"/>
-      <c r="BW7" s="67"/>
-      <c r="BX7" s="67"/>
-      <c r="BY7" s="67"/>
-      <c r="BZ7" s="67"/>
-      <c r="CA7" s="68"/>
-      <c r="CB7" s="64" t="s">
+      <c r="BI7" s="50"/>
+      <c r="BJ7" s="62"/>
+      <c r="BK7" s="62"/>
+      <c r="BL7" s="62"/>
+      <c r="BM7" s="62"/>
+      <c r="BN7" s="62"/>
+      <c r="BO7" s="62"/>
+      <c r="BP7" s="62"/>
+      <c r="BQ7" s="62"/>
+      <c r="BR7" s="50"/>
+      <c r="BS7" s="50"/>
+      <c r="BT7" s="62"/>
+      <c r="BU7" s="62"/>
+      <c r="BV7" s="62"/>
+      <c r="BW7" s="62"/>
+      <c r="BX7" s="62"/>
+      <c r="BY7" s="62"/>
+      <c r="BZ7" s="62"/>
+      <c r="CA7" s="63"/>
+      <c r="CB7" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="CC7" s="69"/>
-      <c r="CD7" s="69"/>
-      <c r="CE7" s="69"/>
-      <c r="CF7" s="69"/>
-      <c r="CG7" s="69"/>
-      <c r="CH7" s="69"/>
-      <c r="CI7" s="69"/>
-      <c r="CJ7" s="69"/>
-      <c r="CK7" s="69"/>
-      <c r="CL7" s="69"/>
-      <c r="CM7" s="69"/>
-      <c r="CN7" s="69"/>
-      <c r="CO7" s="69"/>
-      <c r="CP7" s="69"/>
-      <c r="CQ7" s="69"/>
-      <c r="CR7" s="69"/>
-      <c r="CS7" s="69"/>
-      <c r="CT7" s="69"/>
-      <c r="CU7" s="70"/>
+      <c r="CC7" s="46"/>
+      <c r="CD7" s="46"/>
+      <c r="CE7" s="46"/>
+      <c r="CF7" s="46"/>
+      <c r="CG7" s="46"/>
+      <c r="CH7" s="46"/>
+      <c r="CI7" s="46"/>
+      <c r="CJ7" s="46"/>
+      <c r="CK7" s="46"/>
+      <c r="CL7" s="46"/>
+      <c r="CM7" s="46"/>
+      <c r="CN7" s="46"/>
+      <c r="CO7" s="46"/>
+      <c r="CP7" s="46"/>
+      <c r="CQ7" s="46"/>
+      <c r="CR7" s="46"/>
+      <c r="CS7" s="46"/>
+      <c r="CT7" s="46"/>
+      <c r="CU7" s="47"/>
     </row>
     <row r="8" spans="2:99" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="13" t="s">
@@ -1469,7 +1459,7 @@
         <v>17</v>
       </c>
       <c r="J8" s="16" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="K8" s="12"/>
       <c r="L8" s="12"/>
@@ -1482,10 +1472,10 @@
       <c r="Q8" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="T8" s="52" t="s">
+      <c r="T8" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="U8" s="53" t="s">
+      <c r="U8" s="43" t="s">
         <v>23</v>
       </c>
       <c r="V8" s="54"/>
@@ -1496,7 +1486,7 @@
       <c r="AA8" s="54"/>
       <c r="AB8" s="54"/>
       <c r="AC8" s="54"/>
-      <c r="AD8" s="53" t="s">
+      <c r="AD8" s="43" t="s">
         <v>18</v>
       </c>
       <c r="AE8" s="54"/>
@@ -1508,10 +1498,10 @@
       <c r="AK8" s="54"/>
       <c r="AL8" s="54"/>
       <c r="AM8" s="55"/>
-      <c r="AN8" s="52" t="s">
+      <c r="AN8" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="AO8" s="53" t="s">
+      <c r="AO8" s="43" t="s">
         <v>23</v>
       </c>
       <c r="AP8" s="54"/>
@@ -1522,7 +1512,7 @@
       <c r="AU8" s="54"/>
       <c r="AV8" s="54"/>
       <c r="AW8" s="54"/>
-      <c r="AX8" s="53" t="s">
+      <c r="AX8" s="43" t="s">
         <v>18</v>
       </c>
       <c r="AY8" s="54"/>
@@ -1534,58 +1524,58 @@
       <c r="BE8" s="54"/>
       <c r="BF8" s="54"/>
       <c r="BG8" s="55"/>
-      <c r="BH8" s="52" t="s">
+      <c r="BH8" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="BI8" s="53" t="s">
+      <c r="BI8" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="BJ8" s="62"/>
-      <c r="BK8" s="62"/>
-      <c r="BL8" s="62"/>
-      <c r="BM8" s="62"/>
-      <c r="BN8" s="62"/>
-      <c r="BO8" s="62"/>
-      <c r="BP8" s="62"/>
-      <c r="BQ8" s="62"/>
-      <c r="BR8" s="53" t="s">
+      <c r="BJ8" s="67"/>
+      <c r="BK8" s="67"/>
+      <c r="BL8" s="67"/>
+      <c r="BM8" s="67"/>
+      <c r="BN8" s="67"/>
+      <c r="BO8" s="67"/>
+      <c r="BP8" s="67"/>
+      <c r="BQ8" s="67"/>
+      <c r="BR8" s="43" t="s">
         <v>18</v>
       </c>
       <c r="BS8" s="54"/>
-      <c r="BT8" s="62"/>
-      <c r="BU8" s="62"/>
-      <c r="BV8" s="62"/>
-      <c r="BW8" s="62"/>
-      <c r="BX8" s="62"/>
-      <c r="BY8" s="62"/>
-      <c r="BZ8" s="62"/>
-      <c r="CA8" s="44"/>
-      <c r="CB8" s="52" t="s">
+      <c r="BT8" s="67"/>
+      <c r="BU8" s="67"/>
+      <c r="BV8" s="67"/>
+      <c r="BW8" s="67"/>
+      <c r="BX8" s="67"/>
+      <c r="BY8" s="67"/>
+      <c r="BZ8" s="67"/>
+      <c r="CA8" s="58"/>
+      <c r="CB8" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="CC8" s="53" t="s">
+      <c r="CC8" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="CD8" s="53"/>
-      <c r="CE8" s="53"/>
-      <c r="CF8" s="53"/>
-      <c r="CG8" s="53"/>
-      <c r="CH8" s="53"/>
-      <c r="CI8" s="53"/>
-      <c r="CJ8" s="53"/>
-      <c r="CK8" s="53"/>
-      <c r="CL8" s="53" t="s">
+      <c r="CD8" s="43"/>
+      <c r="CE8" s="43"/>
+      <c r="CF8" s="43"/>
+      <c r="CG8" s="43"/>
+      <c r="CH8" s="43"/>
+      <c r="CI8" s="43"/>
+      <c r="CJ8" s="43"/>
+      <c r="CK8" s="43"/>
+      <c r="CL8" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="CM8" s="53"/>
-      <c r="CN8" s="53"/>
-      <c r="CO8" s="53"/>
-      <c r="CP8" s="53"/>
-      <c r="CQ8" s="53"/>
-      <c r="CR8" s="53"/>
-      <c r="CS8" s="53"/>
-      <c r="CT8" s="53"/>
-      <c r="CU8" s="63"/>
+      <c r="CM8" s="43"/>
+      <c r="CN8" s="43"/>
+      <c r="CO8" s="43"/>
+      <c r="CP8" s="43"/>
+      <c r="CQ8" s="43"/>
+      <c r="CR8" s="43"/>
+      <c r="CS8" s="43"/>
+      <c r="CT8" s="43"/>
+      <c r="CU8" s="44"/>
     </row>
     <row r="9" spans="2:99" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="18" t="s">
@@ -1629,241 +1619,241 @@
         <f>[1]Schedule!D15</f>
         <v>12</v>
       </c>
-      <c r="T9" s="52" t="s">
+      <c r="T9" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="U9" s="56">
+      <c r="U9" s="12">
         <v>7</v>
       </c>
-      <c r="V9" s="56">
+      <c r="V9" s="12">
         <v>15</v>
       </c>
-      <c r="W9" s="56">
-        <v>5</v>
-      </c>
-      <c r="X9" s="56">
+      <c r="W9" s="12">
+        <v>5</v>
+      </c>
+      <c r="X9" s="12">
         <v>13</v>
       </c>
-      <c r="Y9" s="56">
-        <v>3</v>
-      </c>
-      <c r="Z9" s="56">
+      <c r="Y9" s="12">
+        <v>3</v>
+      </c>
+      <c r="Z9" s="12">
         <v>11</v>
       </c>
-      <c r="AA9" s="56">
+      <c r="AA9" s="12">
         <v>17</v>
       </c>
-      <c r="AB9" s="56">
+      <c r="AB9" s="12">
         <v>9</v>
       </c>
-      <c r="AC9" s="56">
-        <v>1</v>
-      </c>
-      <c r="AD9" s="57" t="s">
+      <c r="AC9" s="12">
+        <v>1</v>
+      </c>
+      <c r="AD9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="AE9" s="56">
-        <v>4</v>
-      </c>
-      <c r="AF9" s="56">
+      <c r="AE9" s="12">
+        <v>4</v>
+      </c>
+      <c r="AF9" s="12">
         <v>12</v>
       </c>
-      <c r="AG9" s="56">
+      <c r="AG9" s="12">
         <v>14</v>
       </c>
-      <c r="AH9" s="56">
+      <c r="AH9" s="12">
         <v>6</v>
       </c>
-      <c r="AI9" s="56">
+      <c r="AI9" s="12">
         <v>16</v>
       </c>
-      <c r="AJ9" s="56">
+      <c r="AJ9" s="12">
         <v>8</v>
       </c>
-      <c r="AK9" s="56">
+      <c r="AK9" s="12">
         <v>18</v>
       </c>
-      <c r="AL9" s="56">
+      <c r="AL9" s="12">
         <v>2</v>
       </c>
       <c r="AM9" s="26">
         <v>10</v>
       </c>
-      <c r="AN9" s="52" t="s">
+      <c r="AN9" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="AO9" s="56">
+      <c r="AO9" s="12">
         <v>7</v>
       </c>
-      <c r="AP9" s="56">
+      <c r="AP9" s="12">
         <v>17</v>
       </c>
-      <c r="AQ9" s="56">
+      <c r="AQ9" s="12">
         <v>15</v>
       </c>
-      <c r="AR9" s="56">
-        <v>1</v>
-      </c>
-      <c r="AS9" s="56">
+      <c r="AR9" s="12">
+        <v>1</v>
+      </c>
+      <c r="AS9" s="12">
         <v>11</v>
       </c>
-      <c r="AT9" s="56">
+      <c r="AT9" s="12">
         <v>9</v>
       </c>
-      <c r="AU9" s="56">
+      <c r="AU9" s="12">
         <v>13</v>
       </c>
-      <c r="AV9" s="56">
-        <v>5</v>
-      </c>
-      <c r="AW9" s="56">
-        <v>3</v>
-      </c>
-      <c r="AX9" s="57" t="s">
+      <c r="AV9" s="12">
+        <v>5</v>
+      </c>
+      <c r="AW9" s="12">
+        <v>3</v>
+      </c>
+      <c r="AX9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="AY9" s="56">
+      <c r="AY9" s="12">
         <v>14</v>
       </c>
-      <c r="AZ9" s="56">
+      <c r="AZ9" s="12">
         <v>8</v>
       </c>
-      <c r="BA9" s="56">
+      <c r="BA9" s="12">
         <v>6</v>
       </c>
-      <c r="BB9" s="56">
-        <v>4</v>
-      </c>
-      <c r="BC9" s="56">
+      <c r="BB9" s="12">
+        <v>4</v>
+      </c>
+      <c r="BC9" s="12">
         <v>16</v>
       </c>
-      <c r="BD9" s="56">
+      <c r="BD9" s="12">
         <v>2</v>
       </c>
-      <c r="BE9" s="56">
+      <c r="BE9" s="12">
         <v>10</v>
       </c>
-      <c r="BF9" s="56">
+      <c r="BF9" s="12">
         <v>12</v>
       </c>
       <c r="BG9" s="26">
         <v>18</v>
       </c>
-      <c r="BH9" s="52" t="s">
+      <c r="BH9" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="BI9" s="56">
+      <c r="BI9" s="12">
         <v>7</v>
       </c>
-      <c r="BJ9" s="56">
-        <v>3</v>
-      </c>
-      <c r="BK9" s="56">
+      <c r="BJ9" s="12">
+        <v>3</v>
+      </c>
+      <c r="BK9" s="12">
         <v>13</v>
       </c>
-      <c r="BL9" s="56">
+      <c r="BL9" s="12">
         <v>9</v>
       </c>
-      <c r="BM9" s="56">
+      <c r="BM9" s="12">
         <v>11</v>
       </c>
-      <c r="BN9" s="56">
+      <c r="BN9" s="12">
         <v>15</v>
       </c>
-      <c r="BO9" s="56">
-        <v>1</v>
-      </c>
-      <c r="BP9" s="56">
-        <v>5</v>
-      </c>
-      <c r="BQ9" s="56">
+      <c r="BO9" s="12">
+        <v>1</v>
+      </c>
+      <c r="BP9" s="12">
+        <v>5</v>
+      </c>
+      <c r="BQ9" s="12">
         <v>17</v>
       </c>
-      <c r="BR9" s="57" t="s">
+      <c r="BR9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="BS9" s="56">
+      <c r="BS9" s="12">
         <v>2</v>
       </c>
-      <c r="BT9" s="56">
+      <c r="BT9" s="12">
         <v>6</v>
       </c>
-      <c r="BU9" s="56">
+      <c r="BU9" s="12">
         <v>12</v>
       </c>
-      <c r="BV9" s="56">
+      <c r="BV9" s="12">
         <v>14</v>
       </c>
-      <c r="BW9" s="56">
+      <c r="BW9" s="12">
         <v>16</v>
       </c>
-      <c r="BX9" s="56">
+      <c r="BX9" s="12">
         <v>18</v>
       </c>
-      <c r="BY9" s="56">
+      <c r="BY9" s="12">
         <v>8</v>
       </c>
-      <c r="BZ9" s="56">
+      <c r="BZ9" s="12">
         <v>4</v>
       </c>
       <c r="CA9" s="26">
         <v>10</v>
       </c>
-      <c r="CB9" s="52" t="s">
+      <c r="CB9" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="CC9" s="56">
+      <c r="CC9" s="12">
         <v>17</v>
       </c>
-      <c r="CD9" s="56">
-        <v>3</v>
-      </c>
-      <c r="CE9" s="56">
+      <c r="CD9" s="12">
+        <v>3</v>
+      </c>
+      <c r="CE9" s="12">
         <v>11</v>
       </c>
-      <c r="CF9" s="56">
+      <c r="CF9" s="12">
         <v>13</v>
       </c>
-      <c r="CG9" s="56">
+      <c r="CG9" s="12">
         <v>7</v>
       </c>
-      <c r="CH9" s="56">
+      <c r="CH9" s="12">
         <v>15</v>
       </c>
-      <c r="CI9" s="56">
+      <c r="CI9" s="12">
         <v>9</v>
       </c>
-      <c r="CJ9" s="56">
-        <v>5</v>
-      </c>
-      <c r="CK9" s="56">
-        <v>1</v>
-      </c>
-      <c r="CL9" s="57" t="s">
+      <c r="CJ9" s="12">
+        <v>5</v>
+      </c>
+      <c r="CK9" s="12">
+        <v>1</v>
+      </c>
+      <c r="CL9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="CM9" s="56">
+      <c r="CM9" s="12">
         <v>16</v>
       </c>
-      <c r="CN9" s="56">
+      <c r="CN9" s="12">
         <v>18</v>
       </c>
-      <c r="CO9" s="56">
+      <c r="CO9" s="12">
         <v>2</v>
       </c>
-      <c r="CP9" s="56">
+      <c r="CP9" s="12">
         <v>14</v>
       </c>
-      <c r="CQ9" s="56">
+      <c r="CQ9" s="12">
         <v>12</v>
       </c>
-      <c r="CR9" s="56">
+      <c r="CR9" s="12">
         <v>8</v>
       </c>
-      <c r="CS9" s="56">
-        <v>4</v>
-      </c>
-      <c r="CT9" s="56">
+      <c r="CS9" s="12">
+        <v>4</v>
+      </c>
+      <c r="CT9" s="12">
         <v>6</v>
       </c>
       <c r="CU9" s="26">
@@ -1880,11 +1870,11 @@
       </c>
       <c r="D10" s="12">
         <f t="array" ref="D10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,D9),$J8="Front 9",INDEX($U$12:$AC$12,1,D9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,D9),$J8="Front 9",INDEX($AO$12:$AW$12,1,D9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,D9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,D9)),$B$2="Emerald Lake",_xlfn.IFS($J8="Back 9",INDEX($CM$12:$CU$12,1,D9),$J8="Front 9",INDEX($CC$12:$CK$12,1,D9)))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E10" s="26">
         <f t="array" ref="E10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,E9),$J8="Front 9",INDEX($U$12:$AC$12,1,E9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,E9),$J8="Front 9",INDEX($AO$12:$AW$12,1,E9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,E9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,E9)),$B$2="Emerald Lake",_xlfn.IFS($J8="Back 9",INDEX($CM$12:$CU$12,1,E9),$J8="Front 9",INDEX($CC$12:$CK$12,1,E9)))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F10" s="27">
         <f t="array" ref="F10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,F9),$J8="Front 9",INDEX($U$12:$AC$12,1,F9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,F9),$J8="Front 9",INDEX($AO$12:$AW$12,1,F9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,F9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,F9)),$B$2="Emerald Lake",_xlfn.IFS($J8="Back 9",INDEX($CM$12:$CU$12,1,F9),$J8="Front 9",INDEX($CC$12:$CK$12,1,F9)))</f>
@@ -1892,7 +1882,7 @@
       </c>
       <c r="G10" s="12">
         <f t="array" ref="G10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,G9),$J8="Front 9",INDEX($U$12:$AC$12,1,G9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,G9),$J8="Front 9",INDEX($AO$12:$AW$12,1,G9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,G9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,G9)),$B$2="Emerald Lake",_xlfn.IFS($J8="Back 9",INDEX($CM$12:$CU$12,1,G9),$J8="Front 9",INDEX($CC$12:$CK$12,1,G9)))</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H10" s="26">
         <f t="array" ref="H10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,H9),$J8="Front 9",INDEX($U$12:$AC$12,1,H9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,H9),$J8="Front 9",INDEX($AO$12:$AW$12,1,H9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,H9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,H9)),$B$2="Emerald Lake",_xlfn.IFS($J8="Back 9",INDEX($CM$12:$CU$12,1,H9),$J8="Front 9",INDEX($CC$12:$CK$12,1,H9)))</f>
@@ -1908,11 +1898,11 @@
       </c>
       <c r="K10" s="26">
         <f t="array" ref="K10">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",INDEX($AE$12:$AM$12,1,K9),$J8="Front 9",INDEX($U$12:$AC$12,1,K9)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",INDEX($AY$12:$BG$12,1,K9),$J8="Front 9",INDEX($AO$12:$AW$12,1,K9)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",INDEX($BS$12:$CA$12,1,K9),$J8="Front 9",INDEX($BI$12:$BQ$12,1,K9)),$B$2="Emerald Lake",_xlfn.IFS($J8="Back 9",INDEX($CM$12:$CU$12,1,K9),$J8="Front 9",INDEX($CC$12:$CK$12,1,K9)))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L10" s="12">
         <f>SUM(C10:K10)</f>
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O10" s="22">
         <v>2</v>
@@ -1924,241 +1914,241 @@
         <f>[1]Schedule!D16</f>
         <v>12</v>
       </c>
-      <c r="T10" s="52" t="s">
+      <c r="T10" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="U10" s="56">
+      <c r="U10" s="12">
         <v>7</v>
       </c>
-      <c r="V10" s="56">
+      <c r="V10" s="12">
         <v>15</v>
       </c>
-      <c r="W10" s="56">
-        <v>5</v>
-      </c>
-      <c r="X10" s="56">
+      <c r="W10" s="12">
+        <v>5</v>
+      </c>
+      <c r="X10" s="12">
         <v>13</v>
       </c>
-      <c r="Y10" s="56">
-        <v>3</v>
-      </c>
-      <c r="Z10" s="56">
+      <c r="Y10" s="12">
+        <v>3</v>
+      </c>
+      <c r="Z10" s="12">
         <v>11</v>
       </c>
-      <c r="AA10" s="56">
+      <c r="AA10" s="12">
         <v>17</v>
       </c>
-      <c r="AB10" s="56">
+      <c r="AB10" s="12">
         <v>9</v>
       </c>
-      <c r="AC10" s="56">
-        <v>1</v>
-      </c>
-      <c r="AD10" s="57" t="s">
+      <c r="AC10" s="12">
+        <v>1</v>
+      </c>
+      <c r="AD10" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AE10" s="56">
-        <v>4</v>
-      </c>
-      <c r="AF10" s="56">
+      <c r="AE10" s="12">
+        <v>4</v>
+      </c>
+      <c r="AF10" s="12">
         <v>12</v>
       </c>
-      <c r="AG10" s="56">
+      <c r="AG10" s="12">
         <v>14</v>
       </c>
-      <c r="AH10" s="56">
+      <c r="AH10" s="12">
         <v>6</v>
       </c>
-      <c r="AI10" s="56">
+      <c r="AI10" s="12">
         <v>16</v>
       </c>
-      <c r="AJ10" s="56">
+      <c r="AJ10" s="12">
         <v>8</v>
       </c>
-      <c r="AK10" s="56">
+      <c r="AK10" s="12">
         <v>18</v>
       </c>
-      <c r="AL10" s="56">
+      <c r="AL10" s="12">
         <v>2</v>
       </c>
       <c r="AM10" s="26">
         <v>10</v>
       </c>
-      <c r="AN10" s="52" t="s">
+      <c r="AN10" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="AO10" s="56">
+      <c r="AO10" s="12">
         <v>7</v>
       </c>
-      <c r="AP10" s="56">
+      <c r="AP10" s="12">
         <v>17</v>
       </c>
-      <c r="AQ10" s="56">
+      <c r="AQ10" s="12">
         <v>15</v>
       </c>
-      <c r="AR10" s="56">
-        <v>1</v>
-      </c>
-      <c r="AS10" s="56">
+      <c r="AR10" s="12">
+        <v>1</v>
+      </c>
+      <c r="AS10" s="12">
         <v>11</v>
       </c>
-      <c r="AT10" s="56">
+      <c r="AT10" s="12">
         <v>9</v>
       </c>
-      <c r="AU10" s="56">
+      <c r="AU10" s="12">
         <v>13</v>
       </c>
-      <c r="AV10" s="56">
-        <v>5</v>
-      </c>
-      <c r="AW10" s="56">
-        <v>3</v>
-      </c>
-      <c r="AX10" s="57" t="s">
+      <c r="AV10" s="12">
+        <v>5</v>
+      </c>
+      <c r="AW10" s="12">
+        <v>3</v>
+      </c>
+      <c r="AX10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AY10" s="56">
+      <c r="AY10" s="12">
         <v>14</v>
       </c>
-      <c r="AZ10" s="56">
+      <c r="AZ10" s="12">
         <v>8</v>
       </c>
-      <c r="BA10" s="56">
+      <c r="BA10" s="12">
         <v>6</v>
       </c>
-      <c r="BB10" s="56">
-        <v>4</v>
-      </c>
-      <c r="BC10" s="56">
+      <c r="BB10" s="12">
+        <v>4</v>
+      </c>
+      <c r="BC10" s="12">
         <v>16</v>
       </c>
-      <c r="BD10" s="56">
+      <c r="BD10" s="12">
         <v>2</v>
       </c>
-      <c r="BE10" s="56">
+      <c r="BE10" s="12">
         <v>10</v>
       </c>
-      <c r="BF10" s="56">
+      <c r="BF10" s="12">
         <v>12</v>
       </c>
       <c r="BG10" s="26">
         <v>18</v>
       </c>
-      <c r="BH10" s="52" t="s">
+      <c r="BH10" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="BI10" s="56">
+      <c r="BI10" s="12">
         <v>7</v>
       </c>
-      <c r="BJ10" s="56">
-        <v>3</v>
-      </c>
-      <c r="BK10" s="56">
+      <c r="BJ10" s="12">
+        <v>3</v>
+      </c>
+      <c r="BK10" s="12">
         <v>13</v>
       </c>
-      <c r="BL10" s="56">
+      <c r="BL10" s="12">
         <v>9</v>
       </c>
-      <c r="BM10" s="56">
+      <c r="BM10" s="12">
         <v>11</v>
       </c>
-      <c r="BN10" s="56">
+      <c r="BN10" s="12">
         <v>15</v>
       </c>
-      <c r="BO10" s="56">
-        <v>1</v>
-      </c>
-      <c r="BP10" s="56">
-        <v>5</v>
-      </c>
-      <c r="BQ10" s="56">
+      <c r="BO10" s="12">
+        <v>1</v>
+      </c>
+      <c r="BP10" s="12">
+        <v>5</v>
+      </c>
+      <c r="BQ10" s="12">
         <v>17</v>
       </c>
-      <c r="BR10" s="57" t="s">
+      <c r="BR10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="BS10" s="56">
+      <c r="BS10" s="12">
         <v>2</v>
       </c>
-      <c r="BT10" s="56">
+      <c r="BT10" s="12">
         <v>6</v>
       </c>
-      <c r="BU10" s="56">
+      <c r="BU10" s="12">
         <v>12</v>
       </c>
-      <c r="BV10" s="56">
+      <c r="BV10" s="12">
         <v>14</v>
       </c>
-      <c r="BW10" s="56">
+      <c r="BW10" s="12">
         <v>16</v>
       </c>
-      <c r="BX10" s="56">
+      <c r="BX10" s="12">
         <v>18</v>
       </c>
-      <c r="BY10" s="56">
+      <c r="BY10" s="12">
         <v>8</v>
       </c>
-      <c r="BZ10" s="56">
+      <c r="BZ10" s="12">
         <v>4</v>
       </c>
       <c r="CA10" s="26">
         <v>10</v>
       </c>
-      <c r="CB10" s="52" t="s">
+      <c r="CB10" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="CC10" s="56">
+      <c r="CC10" s="12">
         <v>17</v>
       </c>
-      <c r="CD10" s="56">
-        <v>3</v>
-      </c>
-      <c r="CE10" s="56">
+      <c r="CD10" s="12">
+        <v>3</v>
+      </c>
+      <c r="CE10" s="12">
         <v>11</v>
       </c>
-      <c r="CF10" s="56">
+      <c r="CF10" s="12">
         <v>13</v>
       </c>
-      <c r="CG10" s="56">
+      <c r="CG10" s="12">
         <v>7</v>
       </c>
-      <c r="CH10" s="56">
+      <c r="CH10" s="12">
         <v>15</v>
       </c>
-      <c r="CI10" s="56">
+      <c r="CI10" s="12">
         <v>9</v>
       </c>
-      <c r="CJ10" s="56">
-        <v>5</v>
-      </c>
-      <c r="CK10" s="56">
-        <v>1</v>
-      </c>
-      <c r="CL10" s="57" t="s">
+      <c r="CJ10" s="12">
+        <v>5</v>
+      </c>
+      <c r="CK10" s="12">
+        <v>1</v>
+      </c>
+      <c r="CL10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="CM10" s="56">
+      <c r="CM10" s="12">
         <v>16</v>
       </c>
-      <c r="CN10" s="56">
+      <c r="CN10" s="12">
         <v>18</v>
       </c>
-      <c r="CO10" s="56">
+      <c r="CO10" s="12">
         <v>2</v>
       </c>
-      <c r="CP10" s="56">
+      <c r="CP10" s="12">
         <v>14</v>
       </c>
-      <c r="CQ10" s="56">
+      <c r="CQ10" s="12">
         <v>12</v>
       </c>
-      <c r="CR10" s="56">
+      <c r="CR10" s="12">
         <v>8</v>
       </c>
-      <c r="CS10" s="56">
-        <v>4</v>
-      </c>
-      <c r="CT10" s="56">
+      <c r="CS10" s="12">
+        <v>4</v>
+      </c>
+      <c r="CT10" s="12">
         <v>6</v>
       </c>
       <c r="CU10" s="26">
@@ -2171,39 +2161,39 @@
       </c>
       <c r="C11" s="12">
         <f t="array" ref="C11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$CL$9:$CU$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="D11" s="12">
         <f t="array" ref="D11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$CL$9:$CU$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E11" s="26">
         <f t="array" ref="E11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$CL$9:$CU$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F11" s="27">
         <f t="array" ref="F11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$CL$9:$CU$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="G11" s="12">
         <f t="array" ref="G11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$CL$9:$CU$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="H11" s="26">
         <f t="array" ref="H11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$CL$9:$CU$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="I11" s="27">
         <f t="array" ref="I11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$CL$9:$CU$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="J11" s="12">
         <f t="array" ref="J11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$CL$9:$CU$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K11" s="26">
         <f t="array" ref="K11">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AD$9:$AM$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$AX$9:$BG$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$BR$9:$CA$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J8="Back 9",VLOOKUP($G8,$CL$9:$CU$11,COLUMN()-1,0),$J8="Front 9",VLOOKUP($G8,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="L11" s="12"/>
       <c r="O11" s="22">
@@ -2217,241 +2207,241 @@
         <f>[1]Schedule!D17</f>
         <v>15</v>
       </c>
-      <c r="T11" s="52" t="s">
+      <c r="T11" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="U11" s="56">
+      <c r="U11" s="12">
         <v>17</v>
       </c>
-      <c r="V11" s="56">
+      <c r="V11" s="12">
         <v>9</v>
       </c>
-      <c r="W11" s="56">
-        <v>5</v>
-      </c>
-      <c r="X11" s="56">
+      <c r="W11" s="12">
+        <v>5</v>
+      </c>
+      <c r="X11" s="12">
         <v>7</v>
       </c>
-      <c r="Y11" s="56">
-        <v>3</v>
-      </c>
-      <c r="Z11" s="56">
+      <c r="Y11" s="12">
+        <v>3</v>
+      </c>
+      <c r="Z11" s="12">
         <v>15</v>
       </c>
-      <c r="AA11" s="56">
+      <c r="AA11" s="12">
         <v>11</v>
       </c>
-      <c r="AB11" s="56">
+      <c r="AB11" s="12">
         <v>13</v>
       </c>
-      <c r="AC11" s="56">
-        <v>1</v>
-      </c>
-      <c r="AD11" s="57" t="s">
+      <c r="AC11" s="12">
+        <v>1</v>
+      </c>
+      <c r="AD11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="AE11" s="56">
-        <v>4</v>
-      </c>
-      <c r="AF11" s="56">
+      <c r="AE11" s="12">
+        <v>4</v>
+      </c>
+      <c r="AF11" s="12">
         <v>10</v>
       </c>
-      <c r="AG11" s="56">
+      <c r="AG11" s="12">
         <v>14</v>
       </c>
-      <c r="AH11" s="56">
+      <c r="AH11" s="12">
         <v>6</v>
       </c>
-      <c r="AI11" s="56">
+      <c r="AI11" s="12">
         <v>16</v>
       </c>
-      <c r="AJ11" s="56">
+      <c r="AJ11" s="12">
         <v>12</v>
       </c>
-      <c r="AK11" s="56">
+      <c r="AK11" s="12">
         <v>18</v>
       </c>
-      <c r="AL11" s="56">
+      <c r="AL11" s="12">
         <v>2</v>
       </c>
       <c r="AM11" s="26">
         <v>8</v>
       </c>
-      <c r="AN11" s="52" t="s">
+      <c r="AN11" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="AO11" s="56">
+      <c r="AO11" s="12">
         <v>7</v>
       </c>
-      <c r="AP11" s="56">
+      <c r="AP11" s="12">
         <v>17</v>
       </c>
-      <c r="AQ11" s="56">
+      <c r="AQ11" s="12">
         <v>15</v>
       </c>
-      <c r="AR11" s="56">
-        <v>1</v>
-      </c>
-      <c r="AS11" s="56">
+      <c r="AR11" s="12">
+        <v>1</v>
+      </c>
+      <c r="AS11" s="12">
         <v>11</v>
       </c>
-      <c r="AT11" s="56">
+      <c r="AT11" s="12">
         <v>9</v>
       </c>
-      <c r="AU11" s="56">
+      <c r="AU11" s="12">
         <v>13</v>
       </c>
-      <c r="AV11" s="56">
-        <v>5</v>
-      </c>
-      <c r="AW11" s="56">
-        <v>3</v>
-      </c>
-      <c r="AX11" s="57" t="s">
+      <c r="AV11" s="12">
+        <v>5</v>
+      </c>
+      <c r="AW11" s="12">
+        <v>3</v>
+      </c>
+      <c r="AX11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="AY11" s="56">
+      <c r="AY11" s="12">
         <v>14</v>
       </c>
-      <c r="AZ11" s="56">
+      <c r="AZ11" s="12">
         <v>8</v>
       </c>
-      <c r="BA11" s="56">
+      <c r="BA11" s="12">
         <v>6</v>
       </c>
-      <c r="BB11" s="56">
-        <v>4</v>
-      </c>
-      <c r="BC11" s="56">
+      <c r="BB11" s="12">
+        <v>4</v>
+      </c>
+      <c r="BC11" s="12">
         <v>16</v>
       </c>
-      <c r="BD11" s="56">
+      <c r="BD11" s="12">
         <v>2</v>
       </c>
-      <c r="BE11" s="56">
+      <c r="BE11" s="12">
         <v>10</v>
       </c>
-      <c r="BF11" s="56">
+      <c r="BF11" s="12">
         <v>12</v>
       </c>
       <c r="BG11" s="26">
         <v>18</v>
       </c>
-      <c r="BH11" s="52" t="s">
+      <c r="BH11" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="BI11" s="56">
+      <c r="BI11" s="12">
         <v>7</v>
       </c>
-      <c r="BJ11" s="56">
-        <v>3</v>
-      </c>
-      <c r="BK11" s="56">
+      <c r="BJ11" s="12">
+        <v>3</v>
+      </c>
+      <c r="BK11" s="12">
         <v>13</v>
       </c>
-      <c r="BL11" s="56">
+      <c r="BL11" s="12">
         <v>9</v>
       </c>
-      <c r="BM11" s="56">
+      <c r="BM11" s="12">
         <v>11</v>
       </c>
-      <c r="BN11" s="56">
+      <c r="BN11" s="12">
         <v>15</v>
       </c>
-      <c r="BO11" s="56">
-        <v>1</v>
-      </c>
-      <c r="BP11" s="56">
-        <v>5</v>
-      </c>
-      <c r="BQ11" s="56">
+      <c r="BO11" s="12">
+        <v>1</v>
+      </c>
+      <c r="BP11" s="12">
+        <v>5</v>
+      </c>
+      <c r="BQ11" s="12">
         <v>17</v>
       </c>
-      <c r="BR11" s="57" t="s">
+      <c r="BR11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="BS11" s="56">
+      <c r="BS11" s="12">
         <v>2</v>
       </c>
-      <c r="BT11" s="56">
+      <c r="BT11" s="12">
         <v>6</v>
       </c>
-      <c r="BU11" s="56">
+      <c r="BU11" s="12">
         <v>12</v>
       </c>
-      <c r="BV11" s="56">
+      <c r="BV11" s="12">
         <v>14</v>
       </c>
-      <c r="BW11" s="56">
+      <c r="BW11" s="12">
         <v>16</v>
       </c>
-      <c r="BX11" s="56">
+      <c r="BX11" s="12">
         <v>18</v>
       </c>
-      <c r="BY11" s="56">
+      <c r="BY11" s="12">
         <v>8</v>
       </c>
-      <c r="BZ11" s="56">
+      <c r="BZ11" s="12">
         <v>4</v>
       </c>
       <c r="CA11" s="26">
         <v>10</v>
       </c>
-      <c r="CB11" s="52" t="s">
+      <c r="CB11" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="CC11" s="56">
+      <c r="CC11" s="12">
         <v>17</v>
       </c>
-      <c r="CD11" s="56">
-        <v>3</v>
-      </c>
-      <c r="CE11" s="56">
+      <c r="CD11" s="12">
+        <v>3</v>
+      </c>
+      <c r="CE11" s="12">
         <v>11</v>
       </c>
-      <c r="CF11" s="56">
+      <c r="CF11" s="12">
         <v>13</v>
       </c>
-      <c r="CG11" s="56">
+      <c r="CG11" s="12">
         <v>7</v>
       </c>
-      <c r="CH11" s="56">
+      <c r="CH11" s="12">
         <v>15</v>
       </c>
-      <c r="CI11" s="56">
+      <c r="CI11" s="12">
         <v>9</v>
       </c>
-      <c r="CJ11" s="56">
-        <v>5</v>
-      </c>
-      <c r="CK11" s="56">
-        <v>1</v>
-      </c>
-      <c r="CL11" s="57" t="s">
+      <c r="CJ11" s="12">
+        <v>5</v>
+      </c>
+      <c r="CK11" s="12">
+        <v>1</v>
+      </c>
+      <c r="CL11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="CM11" s="56">
+      <c r="CM11" s="12">
         <v>16</v>
       </c>
-      <c r="CN11" s="56">
+      <c r="CN11" s="12">
         <v>18</v>
       </c>
-      <c r="CO11" s="56">
+      <c r="CO11" s="12">
         <v>2</v>
       </c>
-      <c r="CP11" s="56">
+      <c r="CP11" s="12">
         <v>14</v>
       </c>
-      <c r="CQ11" s="56">
+      <c r="CQ11" s="12">
         <v>12</v>
       </c>
-      <c r="CR11" s="56">
+      <c r="CR11" s="12">
         <v>8</v>
       </c>
-      <c r="CS11" s="56">
-        <v>4</v>
-      </c>
-      <c r="CT11" s="56">
+      <c r="CS11" s="12">
+        <v>4</v>
+      </c>
+      <c r="CT11" s="12">
         <v>6</v>
       </c>
       <c r="CU11" s="26">
@@ -2466,36 +2456,36 @@
         <v>5</v>
       </c>
       <c r="D12" s="30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E12" s="31">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F12" s="29">
         <v>5</v>
       </c>
       <c r="G12" s="30">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H12" s="31">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I12" s="29">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J12" s="30">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K12" s="31">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L12" s="12">
         <f>SUM(C12:K12)</f>
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="M12" s="32">
         <f>SUM(C12:K12)-SUM(C$10:K$10)</f>
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="O12" s="22">
         <v>4</v>
@@ -2507,244 +2497,244 @@
         <f>[1]Schedule!D18</f>
         <v>24</v>
       </c>
-      <c r="T12" s="58" t="s">
+      <c r="T12" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="U12" s="59">
-        <v>4</v>
-      </c>
-      <c r="V12" s="59">
-        <v>3</v>
-      </c>
-      <c r="W12" s="59">
-        <v>4</v>
-      </c>
-      <c r="X12" s="59">
-        <v>5</v>
-      </c>
-      <c r="Y12" s="59">
-        <v>4</v>
-      </c>
-      <c r="Z12" s="59">
-        <v>4</v>
-      </c>
-      <c r="AA12" s="59">
-        <v>3</v>
-      </c>
-      <c r="AB12" s="59">
-        <v>5</v>
-      </c>
-      <c r="AC12" s="59">
-        <v>4</v>
-      </c>
-      <c r="AD12" s="60" t="s">
+      <c r="U12" s="40">
+        <v>4</v>
+      </c>
+      <c r="V12" s="40">
+        <v>3</v>
+      </c>
+      <c r="W12" s="40">
+        <v>4</v>
+      </c>
+      <c r="X12" s="40">
+        <v>5</v>
+      </c>
+      <c r="Y12" s="40">
+        <v>4</v>
+      </c>
+      <c r="Z12" s="40">
+        <v>4</v>
+      </c>
+      <c r="AA12" s="40">
+        <v>3</v>
+      </c>
+      <c r="AB12" s="40">
+        <v>5</v>
+      </c>
+      <c r="AC12" s="40">
+        <v>4</v>
+      </c>
+      <c r="AD12" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="AE12" s="59">
-        <v>4</v>
-      </c>
-      <c r="AF12" s="59">
-        <v>5</v>
-      </c>
-      <c r="AG12" s="59">
-        <v>4</v>
-      </c>
-      <c r="AH12" s="59">
-        <v>4</v>
-      </c>
-      <c r="AI12" s="59">
-        <v>3</v>
-      </c>
-      <c r="AJ12" s="59">
-        <v>4</v>
-      </c>
-      <c r="AK12" s="59">
-        <v>3</v>
-      </c>
-      <c r="AL12" s="59">
-        <v>4</v>
-      </c>
-      <c r="AM12" s="61">
-        <v>5</v>
-      </c>
-      <c r="AN12" s="58" t="s">
+      <c r="AE12" s="40">
+        <v>4</v>
+      </c>
+      <c r="AF12" s="40">
+        <v>5</v>
+      </c>
+      <c r="AG12" s="40">
+        <v>4</v>
+      </c>
+      <c r="AH12" s="40">
+        <v>4</v>
+      </c>
+      <c r="AI12" s="40">
+        <v>3</v>
+      </c>
+      <c r="AJ12" s="40">
+        <v>4</v>
+      </c>
+      <c r="AK12" s="40">
+        <v>3</v>
+      </c>
+      <c r="AL12" s="40">
+        <v>4</v>
+      </c>
+      <c r="AM12" s="42">
+        <v>5</v>
+      </c>
+      <c r="AN12" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="AO12" s="59">
-        <v>4</v>
-      </c>
-      <c r="AP12" s="59">
-        <v>5</v>
-      </c>
-      <c r="AQ12" s="59">
-        <v>3</v>
-      </c>
-      <c r="AR12" s="59">
-        <v>4</v>
-      </c>
-      <c r="AS12" s="59">
-        <v>4</v>
-      </c>
-      <c r="AT12" s="59">
-        <v>3</v>
-      </c>
-      <c r="AU12" s="59">
-        <v>5</v>
-      </c>
-      <c r="AV12" s="59">
-        <v>4</v>
-      </c>
-      <c r="AW12" s="59">
-        <v>4</v>
-      </c>
-      <c r="AX12" s="60" t="s">
+      <c r="AO12" s="40">
+        <v>4</v>
+      </c>
+      <c r="AP12" s="40">
+        <v>5</v>
+      </c>
+      <c r="AQ12" s="40">
+        <v>3</v>
+      </c>
+      <c r="AR12" s="40">
+        <v>4</v>
+      </c>
+      <c r="AS12" s="40">
+        <v>4</v>
+      </c>
+      <c r="AT12" s="40">
+        <v>3</v>
+      </c>
+      <c r="AU12" s="40">
+        <v>5</v>
+      </c>
+      <c r="AV12" s="40">
+        <v>4</v>
+      </c>
+      <c r="AW12" s="40">
+        <v>4</v>
+      </c>
+      <c r="AX12" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="AY12" s="59">
-        <v>4</v>
-      </c>
-      <c r="AZ12" s="59">
-        <v>3</v>
-      </c>
-      <c r="BA12" s="59">
-        <v>5</v>
-      </c>
-      <c r="BB12" s="59">
-        <v>4</v>
-      </c>
-      <c r="BC12" s="59">
-        <v>4</v>
-      </c>
-      <c r="BD12" s="59">
-        <v>4</v>
-      </c>
-      <c r="BE12" s="59">
-        <v>4</v>
-      </c>
-      <c r="BF12" s="59">
-        <v>3</v>
-      </c>
-      <c r="BG12" s="61">
-        <v>5</v>
-      </c>
-      <c r="BH12" s="58" t="s">
+      <c r="AY12" s="40">
+        <v>4</v>
+      </c>
+      <c r="AZ12" s="40">
+        <v>3</v>
+      </c>
+      <c r="BA12" s="40">
+        <v>5</v>
+      </c>
+      <c r="BB12" s="40">
+        <v>4</v>
+      </c>
+      <c r="BC12" s="40">
+        <v>4</v>
+      </c>
+      <c r="BD12" s="40">
+        <v>4</v>
+      </c>
+      <c r="BE12" s="40">
+        <v>4</v>
+      </c>
+      <c r="BF12" s="40">
+        <v>3</v>
+      </c>
+      <c r="BG12" s="42">
+        <v>5</v>
+      </c>
+      <c r="BH12" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="BI12" s="59">
-        <v>5</v>
-      </c>
-      <c r="BJ12" s="59">
-        <v>4</v>
-      </c>
-      <c r="BK12" s="59">
-        <v>3</v>
-      </c>
-      <c r="BL12" s="59">
-        <v>5</v>
-      </c>
-      <c r="BM12" s="59">
-        <v>4</v>
-      </c>
-      <c r="BN12" s="59">
-        <v>3</v>
-      </c>
-      <c r="BO12" s="59">
-        <v>4</v>
-      </c>
-      <c r="BP12" s="59">
-        <v>3</v>
-      </c>
-      <c r="BQ12" s="59">
-        <v>4</v>
-      </c>
-      <c r="BR12" s="60" t="s">
+      <c r="BI12" s="40">
+        <v>5</v>
+      </c>
+      <c r="BJ12" s="40">
+        <v>4</v>
+      </c>
+      <c r="BK12" s="40">
+        <v>3</v>
+      </c>
+      <c r="BL12" s="40">
+        <v>5</v>
+      </c>
+      <c r="BM12" s="40">
+        <v>4</v>
+      </c>
+      <c r="BN12" s="40">
+        <v>3</v>
+      </c>
+      <c r="BO12" s="40">
+        <v>4</v>
+      </c>
+      <c r="BP12" s="40">
+        <v>3</v>
+      </c>
+      <c r="BQ12" s="40">
+        <v>4</v>
+      </c>
+      <c r="BR12" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="BS12" s="59">
-        <v>4</v>
-      </c>
-      <c r="BT12" s="59">
-        <v>4</v>
-      </c>
-      <c r="BU12" s="59">
-        <v>3</v>
-      </c>
-      <c r="BV12" s="59">
-        <v>5</v>
-      </c>
-      <c r="BW12" s="59">
-        <v>4</v>
-      </c>
-      <c r="BX12" s="59">
-        <v>4</v>
-      </c>
-      <c r="BY12" s="59">
-        <v>3</v>
-      </c>
-      <c r="BZ12" s="59">
-        <v>5</v>
-      </c>
-      <c r="CA12" s="61">
-        <v>4</v>
-      </c>
-      <c r="CB12" s="58" t="s">
+      <c r="BS12" s="40">
+        <v>4</v>
+      </c>
+      <c r="BT12" s="40">
+        <v>4</v>
+      </c>
+      <c r="BU12" s="40">
+        <v>3</v>
+      </c>
+      <c r="BV12" s="40">
+        <v>5</v>
+      </c>
+      <c r="BW12" s="40">
+        <v>4</v>
+      </c>
+      <c r="BX12" s="40">
+        <v>4</v>
+      </c>
+      <c r="BY12" s="40">
+        <v>3</v>
+      </c>
+      <c r="BZ12" s="40">
+        <v>5</v>
+      </c>
+      <c r="CA12" s="42">
+        <v>4</v>
+      </c>
+      <c r="CB12" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="CC12" s="59">
-        <v>4</v>
-      </c>
-      <c r="CD12" s="59">
-        <v>4</v>
-      </c>
-      <c r="CE12" s="59">
-        <v>3</v>
-      </c>
-      <c r="CF12" s="59">
-        <v>4</v>
-      </c>
-      <c r="CG12" s="59">
-        <v>5</v>
-      </c>
-      <c r="CH12" s="59">
-        <v>4</v>
-      </c>
-      <c r="CI12" s="59">
-        <v>3</v>
-      </c>
-      <c r="CJ12" s="59">
-        <v>4</v>
-      </c>
-      <c r="CK12" s="59">
-        <v>4</v>
-      </c>
-      <c r="CL12" s="60" t="s">
+      <c r="CC12" s="40">
+        <v>4</v>
+      </c>
+      <c r="CD12" s="40">
+        <v>4</v>
+      </c>
+      <c r="CE12" s="40">
+        <v>3</v>
+      </c>
+      <c r="CF12" s="40">
+        <v>4</v>
+      </c>
+      <c r="CG12" s="40">
+        <v>5</v>
+      </c>
+      <c r="CH12" s="40">
+        <v>4</v>
+      </c>
+      <c r="CI12" s="40">
+        <v>3</v>
+      </c>
+      <c r="CJ12" s="40">
+        <v>4</v>
+      </c>
+      <c r="CK12" s="40">
+        <v>4</v>
+      </c>
+      <c r="CL12" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="CM12" s="59">
-        <v>4</v>
-      </c>
-      <c r="CN12" s="59">
-        <v>4</v>
-      </c>
-      <c r="CO12" s="59">
-        <v>4</v>
-      </c>
-      <c r="CP12" s="59">
-        <v>3</v>
-      </c>
-      <c r="CQ12" s="59">
-        <v>5</v>
-      </c>
-      <c r="CR12" s="59">
-        <v>4</v>
-      </c>
-      <c r="CS12" s="59">
-        <v>3</v>
-      </c>
-      <c r="CT12" s="59">
-        <v>4</v>
-      </c>
-      <c r="CU12" s="61">
+      <c r="CM12" s="40">
+        <v>4</v>
+      </c>
+      <c r="CN12" s="40">
+        <v>4</v>
+      </c>
+      <c r="CO12" s="40">
+        <v>4</v>
+      </c>
+      <c r="CP12" s="40">
+        <v>3</v>
+      </c>
+      <c r="CQ12" s="40">
+        <v>5</v>
+      </c>
+      <c r="CR12" s="40">
+        <v>4</v>
+      </c>
+      <c r="CS12" s="40">
+        <v>3</v>
+      </c>
+      <c r="CT12" s="40">
+        <v>4</v>
+      </c>
+      <c r="CU12" s="42">
         <v>5</v>
       </c>
     </row>
@@ -2754,11 +2744,11 @@
       </c>
       <c r="C13" s="27">
         <f t="shared" ref="C13:K13" si="0">INT($D$8/18)+IF(C11&lt;=MOD($D$8,18),1,0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" s="12">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" s="26">
         <f t="shared" si="0"/>
@@ -2766,19 +2756,19 @@
       </c>
       <c r="F13" s="27">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G13" s="12">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H13" s="26">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I13" s="27">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J13" s="12">
         <f t="shared" si="0"/>
@@ -2806,19 +2796,19 @@
       </c>
       <c r="C14" s="27">
         <f>C12-C13</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D14" s="12">
         <f t="shared" ref="D14:K14" si="1">D12-INT($D$8/18)-IF(D11&lt;=MOD($D$8,18),1,0)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E14" s="26">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F14" s="27">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G14" s="12">
         <f t="shared" si="1"/>
@@ -2826,27 +2816,27 @@
       </c>
       <c r="H14" s="26">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I14" s="27">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J14" s="12">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K14" s="26">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L14" s="33">
         <f>SUM(C14:K14)</f>
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="M14" s="32">
         <f>SUM(C14:K14)-SUM(C$10:K$10)</f>
-        <v>-2</v>
+        <v>3</v>
       </c>
       <c r="O14" s="22">
         <v>6</v>
@@ -2869,11 +2859,11 @@
       </c>
       <c r="D15" s="36">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="37">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" s="35">
         <f t="shared" si="2"/>
@@ -2885,19 +2875,19 @@
       </c>
       <c r="H15" s="37">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I15" s="35">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" s="36">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" s="37">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L15" s="12"/>
       <c r="O15" s="22">
@@ -2936,14 +2926,14 @@
     </row>
     <row r="17" spans="2:17" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="13" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C17" s="14" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="12">
         <f>_xlfn.XLOOKUP(B17,$P$9:$P$23,$Q$9:$Q$23)</f>
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="E17" s="12"/>
       <c r="F17" s="12" t="s">
@@ -2958,7 +2948,7 @@
       </c>
       <c r="J17" s="12" t="str">
         <f>J8</f>
-        <v>Front 9</v>
+        <v>Back 9</v>
       </c>
       <c r="K17" s="12"/>
       <c r="L17" s="12"/>
@@ -3027,11 +3017,11 @@
       </c>
       <c r="D19" s="12">
         <f t="array" ref="D19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,D18),$J17="Front 9",INDEX($U$12:$AC$12,1,D18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,D18),$J17="Front 9",INDEX($AO$12:$AW$12,1,D18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,D18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,D18)),$B$2="Emerald Lake",_xlfn.IFS($J17="Back 9",INDEX($CM$12:$CU$12,1,D18),$J17="Front 9",INDEX($CC$12:$CK$12,1,D18)))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E19" s="26">
         <f t="array" ref="E19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,E18),$J17="Front 9",INDEX($U$12:$AC$12,1,E18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,E18),$J17="Front 9",INDEX($AO$12:$AW$12,1,E18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,E18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,E18)),$B$2="Emerald Lake",_xlfn.IFS($J17="Back 9",INDEX($CM$12:$CU$12,1,E18),$J17="Front 9",INDEX($CC$12:$CK$12,1,E18)))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F19" s="27">
         <f t="array" ref="F19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,F18),$J17="Front 9",INDEX($U$12:$AC$12,1,F18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,F18),$J17="Front 9",INDEX($AO$12:$AW$12,1,F18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,F18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,F18)),$B$2="Emerald Lake",_xlfn.IFS($J17="Back 9",INDEX($CM$12:$CU$12,1,F18),$J17="Front 9",INDEX($CC$12:$CK$12,1,F18)))</f>
@@ -3039,7 +3029,7 @@
       </c>
       <c r="G19" s="12">
         <f t="array" ref="G19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,G18),$J17="Front 9",INDEX($U$12:$AC$12,1,G18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,G18),$J17="Front 9",INDEX($AO$12:$AW$12,1,G18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,G18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,G18)),$B$2="Emerald Lake",_xlfn.IFS($J17="Back 9",INDEX($CM$12:$CU$12,1,G18),$J17="Front 9",INDEX($CC$12:$CK$12,1,G18)))</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H19" s="26">
         <f t="array" ref="H19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,H18),$J17="Front 9",INDEX($U$12:$AC$12,1,H18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,H18),$J17="Front 9",INDEX($AO$12:$AW$12,1,H18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,H18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,H18)),$B$2="Emerald Lake",_xlfn.IFS($J17="Back 9",INDEX($CM$12:$CU$12,1,H18),$J17="Front 9",INDEX($CC$12:$CK$12,1,H18)))</f>
@@ -3055,11 +3045,11 @@
       </c>
       <c r="K19" s="26">
         <f t="array" ref="K19">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",INDEX($AE$12:$AM$12,1,K18),$J17="Front 9",INDEX($U$12:$AC$12,1,K18)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",INDEX($AY$12:$BG$12,1,K18),$J17="Front 9",INDEX($AO$12:$AW$12,1,K18)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",INDEX($BS$12:$CA$12,1,K18),$J17="Front 9",INDEX($BI$12:$BQ$12,1,K18)),$B$2="Emerald Lake",_xlfn.IFS($J17="Back 9",INDEX($CM$12:$CU$12,1,K18),$J17="Front 9",INDEX($CC$12:$CK$12,1,K18)))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L19" s="12">
         <f>SUM(C19:K19)</f>
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O19" s="22">
         <f>O18+1</f>
@@ -3079,39 +3069,39 @@
       </c>
       <c r="C20" s="12">
         <f t="array" ref="C20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$CL$9:$CU$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="D20" s="12">
         <f t="array" ref="D20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$CL$9:$CU$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E20" s="26">
         <f t="array" ref="E20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$CL$9:$CU$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F20" s="27">
         <f t="array" ref="F20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$CL$9:$CU$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="G20" s="12">
         <f t="array" ref="G20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$CL$9:$CU$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="H20" s="26">
         <f t="array" ref="H20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$CL$9:$CU$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="I20" s="27">
         <f t="array" ref="I20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$CL$9:$CU$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="J20" s="12">
         <f t="array" ref="J20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$CL$9:$CU$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K20" s="26">
         <f t="array" ref="K20">_xlfn.IFS($B$2="Skybrook",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AD$9:$AM$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$T$9:$AC$11,COLUMN()-1,0)),$B$2="Highland Creek",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$AX$9:$BG$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$AN$9:$AW$11,COLUMN()-1,0)),$B$2="Warrior Golf Club",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$BR$9:$CA$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$BH$9:$BQ$11,COLUMN()-1,0)),$B$2="Emerald Lake",_xlfn.IFS($J17="Back 9",VLOOKUP($G17,$CL$9:$CU$11,COLUMN()-1,0),$J17="Front 9",VLOOKUP($G17,$CB$9:$CK$11,COLUMN()-1,0)))</f>
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="L20" s="12"/>
       <c r="O20" s="22">
@@ -3130,10 +3120,10 @@
         <v>34</v>
       </c>
       <c r="C21" s="29">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D21" s="30">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E21" s="31">
         <v>6</v>
@@ -3142,27 +3132,27 @@
         <v>6</v>
       </c>
       <c r="G21" s="30">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H21" s="31">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I21" s="29">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J21" s="30">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K21" s="31">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="L21" s="12">
         <f>SUM(C21:K21)</f>
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="M21" s="32">
         <f>SUM(C21:K21)-SUM(C$10:K$10)</f>
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="O21" s="22">
         <v>13</v>
@@ -3185,11 +3175,11 @@
       </c>
       <c r="D22" s="12">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E22" s="26">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F22" s="27">
         <f t="shared" si="3"/>
@@ -3197,7 +3187,7 @@
       </c>
       <c r="G22" s="12">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H22" s="26">
         <f t="shared" si="3"/>
@@ -3205,15 +3195,15 @@
       </c>
       <c r="I22" s="27">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J22" s="12">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K22" s="26">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L22" s="32"/>
       <c r="O22" s="22">
@@ -3233,15 +3223,15 @@
       </c>
       <c r="C23" s="27">
         <f t="shared" ref="C23:K23" si="4">C21-C22</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D23" s="12">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E23" s="26">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F23" s="27">
         <f t="shared" si="4"/>
@@ -3249,31 +3239,31 @@
       </c>
       <c r="G23" s="12">
         <f t="shared" si="4"/>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H23" s="26">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I23" s="27">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J23" s="12">
         <f t="shared" si="4"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K23" s="26">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L23" s="33">
         <f>SUM(C23:K23)</f>
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="M23" s="32">
         <f>SUM(C23:K23)-SUM(C$10:K$10)</f>
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="O23" s="22">
         <v>15</v>
@@ -3296,11 +3286,11 @@
       </c>
       <c r="D24" s="36">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" s="37">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F24" s="35">
         <f t="shared" si="5"/>
@@ -3312,7 +3302,7 @@
       </c>
       <c r="H24" s="37">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" s="35">
         <f t="shared" si="5"/>
@@ -3320,33 +3310,33 @@
       </c>
       <c r="J24" s="36">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K24" s="37">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L24" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="CC8:CK8"/>
-    <mergeCell ref="CL8:CU8"/>
-    <mergeCell ref="CB7:CU7"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="T7:AM7"/>
     <mergeCell ref="J1:M1"/>
     <mergeCell ref="AD8:AM8"/>
     <mergeCell ref="AX8:BG8"/>
     <mergeCell ref="AN7:BG7"/>
     <mergeCell ref="L3:M5"/>
     <mergeCell ref="U8:AC8"/>
-    <mergeCell ref="B5:B6"/>
     <mergeCell ref="AO8:AW8"/>
     <mergeCell ref="L2:M2"/>
-    <mergeCell ref="BH7:CA7"/>
     <mergeCell ref="J3:K5"/>
     <mergeCell ref="J2:K2"/>
+    <mergeCell ref="CC8:CK8"/>
+    <mergeCell ref="CL8:CU8"/>
+    <mergeCell ref="CB7:CU7"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="T7:AM7"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="BH7:CA7"/>
     <mergeCell ref="BR8:CA8"/>
     <mergeCell ref="BI8:BQ8"/>
   </mergeCells>

</xml_diff>